<commit_message>
Commission template: fish section
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QC6CoyQvjhDFZcFwnpY687
</commit_message>
<xml_diff>
--- a/cute-pets-dashboard/templates/commissions.xlsx
+++ b/cute-pets-dashboard/templates/commissions.xlsx
@@ -510,6 +510,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -528,7 +529,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>عمولة قسم الأسواق</t>
+          <t>عمولة قسم الأسماك</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -658,6 +659,7 @@
       <c r="D15" s="5" t="n"/>
       <c r="E15" s="5" t="n"/>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
@@ -722,6 +724,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
         <is>
@@ -917,7 +920,7 @@
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="A4:A23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"عمولة مبيعات المتاجر,عمولة منتجات الاستيراد في المحل,عمولة قسم الأسواق,عمولة التوصيل للسواقين"</formula1>
+      <formula1>"عمولة مبيعات المتاجر,عمولة منتجات الاستيراد في المحل,عمولة قسم الأسماك,عمولة التوصيل للسواقين"</formula1>
     </dataValidation>
     <dataValidation sqref="E4:E23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"كامل المبلغ,الزيادة فقط"</formula1>

</xml_diff>